<commit_message>
Requirements file & updated data
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d5cbc24d1a217bff/Poker/Bankroll/stang-gang/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{DC165FDB-1FC4-4119-81A5-A298CFEEDA9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C562163-879E-4A92-B1F8-DD1AF1B79CB1}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{DC165FDB-1FC4-4119-81A5-A298CFEEDA9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9FF460D1-3C78-41D7-BAF1-E4C659C50073}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{A7134671-C15C-4531-A6D4-3327DA0B4BB1}"/>
+    <workbookView xWindow="4668" yWindow="3720" windowWidth="17280" windowHeight="9960" xr2:uid="{A7134671-C15C-4531-A6D4-3327DA0B4BB1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -721,7 +721,7 @@
         <v>46062</v>
       </c>
       <c r="C36">
-        <v>2266</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -729,7 +729,7 @@
         <v>46063</v>
       </c>
       <c r="C37">
-        <v>2562</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -737,7 +737,7 @@
         <v>46065</v>
       </c>
       <c r="C38">
-        <v>2605</v>
+        <v>2505</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -745,7 +745,7 @@
         <v>46066</v>
       </c>
       <c r="C39">
-        <v>2773</v>
+        <v>2673</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -753,7 +753,7 @@
         <v>46068</v>
       </c>
       <c r="C40">
-        <v>2555</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
@@ -761,7 +761,7 @@
         <v>46069</v>
       </c>
       <c r="C41">
-        <v>2506</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -769,7 +769,7 @@
         <v>46070</v>
       </c>
       <c r="C42">
-        <v>2645</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -777,7 +777,7 @@
         <v>46071</v>
       </c>
       <c r="C43">
-        <v>2831</v>
+        <v>2731</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -785,7 +785,7 @@
         <v>46072</v>
       </c>
       <c r="C44">
-        <v>2760</v>
+        <v>2660</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
@@ -793,7 +793,7 @@
         <v>46073</v>
       </c>
       <c r="C45">
-        <v>2590</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
@@ -801,7 +801,7 @@
         <v>46075</v>
       </c>
       <c r="C46">
-        <v>2367</v>
+        <v>2267</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
@@ -809,7 +809,7 @@
         <v>46076</v>
       </c>
       <c r="C47">
-        <v>2660</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
@@ -817,7 +817,7 @@
         <v>46077</v>
       </c>
       <c r="C48">
-        <v>2682</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -825,7 +825,7 @@
         <v>46078</v>
       </c>
       <c r="C49">
-        <v>3096</v>
+        <v>2996</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
@@ -833,7 +833,7 @@
         <v>46079</v>
       </c>
       <c r="C50">
-        <v>3092</v>
+        <v>2992</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
@@ -841,7 +841,7 @@
         <v>46080</v>
       </c>
       <c r="C51">
-        <v>3127</v>
+        <v>3027</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
@@ -849,7 +849,7 @@
         <v>46082</v>
       </c>
       <c r="C52">
-        <v>2845</v>
+        <v>2745</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
@@ -857,7 +857,7 @@
         <v>46083</v>
       </c>
       <c r="C53">
-        <v>2679</v>
+        <v>2579</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
@@ -865,7 +865,7 @@
         <v>46084</v>
       </c>
       <c r="C54">
-        <v>2530</v>
+        <v>2430</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
@@ -873,7 +873,7 @@
         <v>46085</v>
       </c>
       <c r="C55">
-        <v>2370</v>
+        <v>2270</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
@@ -881,7 +881,7 @@
         <v>46086</v>
       </c>
       <c r="C56">
-        <v>2602</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
@@ -889,7 +889,7 @@
         <v>46087</v>
       </c>
       <c r="C57">
-        <v>2546</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
@@ -897,7 +897,7 @@
         <v>46088</v>
       </c>
       <c r="C58">
-        <v>2858</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
@@ -905,7 +905,7 @@
         <v>46089</v>
       </c>
       <c r="C59">
-        <v>3139</v>
+        <v>3039</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
@@ -913,7 +913,7 @@
         <v>46089</v>
       </c>
       <c r="C60">
-        <v>3144</v>
+        <v>3044</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
@@ -921,7 +921,7 @@
         <v>46090</v>
       </c>
       <c r="C61">
-        <v>3406</v>
+        <v>3306</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
@@ -929,7 +929,7 @@
         <v>46091</v>
       </c>
       <c r="C62">
-        <v>3638</v>
+        <v>3538</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
@@ -937,7 +937,7 @@
         <v>46092</v>
       </c>
       <c r="C63">
-        <v>3727</v>
+        <v>3627</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
@@ -948,7 +948,7 @@
         <v>1010</v>
       </c>
       <c r="C64">
-        <v>3702</v>
+        <v>3602</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Profit vs Balance correction for new data
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d5cbc24d1a217bff/Poker/Bankroll/stang-gang/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{DC165FDB-1FC4-4119-81A5-A298CFEEDA9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1B77B6A-1DAC-4141-B8D4-5ED1A201FE78}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{DC165FDB-1FC4-4119-81A5-A298CFEEDA9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FABF5127-4A5D-4FEF-8798-1E63696F2633}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A7134671-C15C-4531-A6D4-3327DA0B4BB1}"/>
+    <workbookView xWindow="3348" yWindow="2916" windowWidth="17280" windowHeight="9960" xr2:uid="{A7134671-C15C-4531-A6D4-3327DA0B4BB1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -956,7 +956,7 @@
         <v>46094</v>
       </c>
       <c r="C65">
-        <v>3955</v>
+        <v>3855</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
@@ -964,7 +964,7 @@
         <v>46095</v>
       </c>
       <c r="C66">
-        <v>4398</v>
+        <v>4298</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
@@ -972,7 +972,7 @@
         <v>46096</v>
       </c>
       <c r="C67">
-        <v>4218</v>
+        <v>4118</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -980,7 +980,7 @@
         <v>46097</v>
       </c>
       <c r="C68">
-        <v>4269</v>
+        <v>4169</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -988,7 +988,7 @@
         <v>46098</v>
       </c>
       <c r="C69">
-        <v>4106</v>
+        <v>4006</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
@@ -996,7 +996,7 @@
         <v>46099</v>
       </c>
       <c r="C70">
-        <v>4458</v>
+        <v>4358</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
@@ -1004,7 +1004,7 @@
         <v>46100</v>
       </c>
       <c r="C71">
-        <v>4251</v>
+        <v>4151</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
@@ -1012,7 +1012,7 @@
         <v>46101</v>
       </c>
       <c r="C72">
-        <v>4249</v>
+        <v>4149</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
@@ -1023,7 +1023,7 @@
         <v>1079</v>
       </c>
       <c r="C73">
-        <v>3956</v>
+        <v>3856</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
@@ -1031,7 +1031,7 @@
         <v>46104</v>
       </c>
       <c r="C74">
-        <v>4484</v>
+        <v>4384</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
@@ -1039,7 +1039,7 @@
         <v>46105</v>
       </c>
       <c r="C75">
-        <v>4474</v>
+        <v>4374</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
@@ -1047,7 +1047,7 @@
         <v>46106</v>
       </c>
       <c r="C76">
-        <v>4686</v>
+        <v>4586</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
@@ -1055,7 +1055,7 @@
         <v>46107</v>
       </c>
       <c r="C77">
-        <v>4408</v>
+        <v>4308</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
@@ -1063,7 +1063,7 @@
         <v>46108</v>
       </c>
       <c r="C78">
-        <v>3970</v>
+        <v>3870</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
@@ -1071,7 +1071,7 @@
         <v>46109</v>
       </c>
       <c r="C79">
-        <v>3905</v>
+        <v>3805</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
@@ -1079,7 +1079,7 @@
         <v>46110</v>
       </c>
       <c r="C80">
-        <v>4435</v>
+        <v>4335</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
@@ -1087,7 +1087,7 @@
         <v>46111</v>
       </c>
       <c r="C81">
-        <v>3998</v>
+        <v>3898</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
@@ -1095,7 +1095,7 @@
         <v>46112</v>
       </c>
       <c r="C82">
-        <v>3717</v>
+        <v>3617</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
@@ -1106,7 +1106,7 @@
         <v>1139</v>
       </c>
       <c r="C83">
-        <v>4104</v>
+        <v>4004</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
@@ -1114,7 +1114,7 @@
         <v>46114</v>
       </c>
       <c r="C84">
-        <v>4304</v>
+        <v>4204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New Data, New Music
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d5cbc24d1a217bff/Poker/Bankroll/stang-gang/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{DC165FDB-1FC4-4119-81A5-A298CFEEDA9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FABF5127-4A5D-4FEF-8798-1E63696F2633}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="13_ncr:1_{DC165FDB-1FC4-4119-81A5-A298CFEEDA9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F6CE7F5-9D5C-4344-AF75-E28A991B14AD}"/>
   <bookViews>
-    <workbookView xWindow="3348" yWindow="2916" windowWidth="17280" windowHeight="9960" xr2:uid="{A7134671-C15C-4531-A6D4-3327DA0B4BB1}"/>
+    <workbookView xWindow="2760" yWindow="3024" windowWidth="17280" windowHeight="9960" xr2:uid="{A7134671-C15C-4531-A6D4-3327DA0B4BB1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -98,10 +98,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -421,7 +417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A52CD65-A2BF-4AC2-8075-EA939B042110}">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -1117,6 +1113,137 @@
         <v>4204</v>
       </c>
     </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" s="1">
+        <v>46115</v>
+      </c>
+      <c r="C85">
+        <v>4883</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" s="1">
+        <v>46116</v>
+      </c>
+      <c r="C86">
+        <v>5339</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" s="1">
+        <v>46117</v>
+      </c>
+      <c r="C87">
+        <v>5563</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" s="1">
+        <v>46118</v>
+      </c>
+      <c r="C88">
+        <v>5750</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" s="1">
+        <v>46119</v>
+      </c>
+      <c r="C89">
+        <v>5666</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" s="1">
+        <v>46120</v>
+      </c>
+      <c r="C90">
+        <v>5701</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" s="1">
+        <v>46121</v>
+      </c>
+      <c r="C91">
+        <v>5508</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92" s="1">
+        <v>46122</v>
+      </c>
+      <c r="C92">
+        <v>5276</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93" s="1">
+        <v>46124</v>
+      </c>
+      <c r="C93">
+        <v>4817</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" s="1">
+        <v>46125</v>
+      </c>
+      <c r="C94">
+        <v>4794</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" s="1">
+        <v>46126</v>
+      </c>
+      <c r="C95">
+        <v>4330</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A96" s="1">
+        <v>46127</v>
+      </c>
+      <c r="C96">
+        <v>3926</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97" s="1">
+        <v>46131</v>
+      </c>
+      <c r="C97">
+        <v>4354</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A98" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C98">
+        <v>4300</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A99" s="1">
+        <v>46133</v>
+      </c>
+      <c r="C99">
+        <v>4496</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100" s="1">
+        <v>46134</v>
+      </c>
+      <c r="B100">
+        <v>1219</v>
+      </c>
+      <c r="C100">
+        <v>4512</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>